<commit_message>
Without LLM Final Model Completed
</commit_message>
<xml_diff>
--- a/With LLM/Intraday_Cross_Sectional_Mean_Reversion_Without_Sentiment/Indian_log_volatile/live_volatiles_results_all_india.xlsx
+++ b/With LLM/Intraday_Cross_Sectional_Mean_Reversion_Without_Sentiment/Indian_log_volatile/live_volatiles_results_all_india.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1097,6 +1097,83 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>-0.11%</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>-0.11%</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>-0.11%</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>-0.11%</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>₹-113.70</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>-24.94%</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>-0.11%</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>-0.11%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>